<commit_message>
Allow blank ID/GPS on extra measurements and scale the brief classification table.
Extra rows inherit plant fields on save; analysis snapshot CSS fits narrow cards. Keep interview prep docs local via gitignore.
</commit_message>
<xml_diff>
--- a/Spicebush.xlsx
+++ b/Spicebush.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,32 +558,32 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1480</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6012</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2025-03</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1522</v>
-      </c>
-      <c r="D4" t="n">
-        <v>6036</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>2.51</v>
-      </c>
       <c r="G4" t="n">
-        <v>2.38</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>2.3</v>
+        <v>3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -594,7 +594,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -602,24 +602,24 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1530</v>
+        <v>1522</v>
       </c>
       <c r="D5" t="n">
-        <v>6005</v>
+        <v>6036</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.18</v>
+        <v>2.51</v>
       </c>
       <c r="G5" t="n">
-        <v>2.11</v>
+        <v>2.38</v>
       </c>
       <c r="H5" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -638,39 +638,35 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1482</v>
+        <v>1530</v>
       </c>
       <c r="D6" t="n">
-        <v>5968</v>
+        <v>6005</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>6.8</v>
+        <v>3.18</v>
       </c>
       <c r="G6" t="n">
-        <v>3.7</v>
+        <v>2.11</v>
       </c>
       <c r="H6" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>also Female</t>
-        </is>
-      </c>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -678,10 +674,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1337</v>
+        <v>1482</v>
       </c>
       <c r="D7" t="n">
-        <v>5908</v>
+        <v>5968</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -689,24 +685,28 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.05</v>
+        <v>6.8</v>
       </c>
       <c r="G7" t="n">
-        <v>1.9</v>
+        <v>3.7</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>also Female</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -714,10 +714,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1577</v>
+        <v>1337</v>
       </c>
       <c r="D8" t="n">
-        <v>5881</v>
+        <v>5908</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -725,24 +725,24 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>13.5</v>
+        <v>3.05</v>
       </c>
       <c r="G8" t="n">
-        <v>5.9</v>
+        <v>1.9</v>
       </c>
       <c r="H8" t="n">
-        <v>6.1</v>
+        <v>2</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -750,35 +750,35 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1600</v>
+        <v>1577</v>
       </c>
       <c r="D9" t="n">
-        <v>5860</v>
+        <v>5881</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>15</v>
+        <v>13.5</v>
       </c>
       <c r="G9" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="H9" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -786,35 +786,35 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1598</v>
+        <v>1600</v>
       </c>
       <c r="D10" t="n">
-        <v>5907</v>
+        <v>5860</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>7.3</v>
+        <v>15</v>
       </c>
       <c r="G10" t="n">
-        <v>4.6</v>
+        <v>5.8</v>
       </c>
       <c r="H10" t="n">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -822,35 +822,35 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1550</v>
+        <v>1598</v>
       </c>
       <c r="D11" t="n">
-        <v>5876</v>
+        <v>5907</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>M</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>F</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -858,10 +858,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1593</v>
+        <v>1550</v>
       </c>
       <c r="D12" t="n">
-        <v>5890</v>
+        <v>5876</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -869,24 +869,24 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1.65</v>
+        <v>8.1</v>
       </c>
       <c r="G12" t="n">
-        <v>1.04</v>
+        <v>3.7</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1526</v>
+        <v>1593</v>
       </c>
       <c r="D13" t="n">
-        <v>5822</v>
+        <v>5890</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -905,13 +905,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>8.699999999999999</v>
+        <v>1.65</v>
       </c>
       <c r="G13" t="n">
-        <v>3.7</v>
+        <v>1.04</v>
       </c>
       <c r="H13" t="n">
-        <v>3.6</v>
+        <v>0.7</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -930,37 +930,35 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1550</v>
+        <v>1526</v>
       </c>
       <c r="D14" t="n">
-        <v>5873</v>
+        <v>5822</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.7</v>
       </c>
       <c r="H14" t="n">
-        <v>0.45</v>
+        <v>3.6</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>U</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -968,18 +966,18 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1554</v>
+        <v>1550</v>
       </c>
       <c r="D15" t="n">
-        <v>5837</v>
+        <v>5873</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -987,7 +985,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.83</v>
+        <v>0.45</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -998,7 +996,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1006,10 +1004,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1523</v>
+        <v>1554</v>
       </c>
       <c r="D16" t="n">
-        <v>5844</v>
+        <v>5837</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1017,24 +1015,26 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G16" t="n">
-        <v>5.9</v>
+        <v>0.8</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H16" t="n">
-        <v>5.1</v>
+        <v>0.83</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1042,10 +1042,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1518</v>
+        <v>1523</v>
       </c>
       <c r="D17" t="n">
-        <v>5865</v>
+        <v>5844</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1053,24 +1053,24 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>7.25</v>
+        <v>10.5</v>
       </c>
       <c r="G17" t="n">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="H17" t="n">
-        <v>5.03</v>
+        <v>5.1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1078,35 +1078,35 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1458</v>
+        <v>1518</v>
       </c>
       <c r="D18" t="n">
-        <v>5809</v>
+        <v>5865</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1.61</v>
+        <v>7.25</v>
       </c>
       <c r="G18" t="n">
-        <v>0.4</v>
+        <v>5.4</v>
       </c>
       <c r="H18" t="n">
-        <v>1.25</v>
+        <v>5.03</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1114,24 +1114,24 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1398</v>
+        <v>1458</v>
       </c>
       <c r="D19" t="n">
-        <v>5870</v>
+        <v>5809</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.26</v>
+        <v>1.61</v>
       </c>
       <c r="G19" t="n">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="H19" t="n">
-        <v>1.75</v>
+        <v>1.25</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1142,7 +1142,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1150,10 +1150,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1350</v>
+        <v>1398</v>
       </c>
       <c r="D20" t="n">
-        <v>5701</v>
+        <v>5870</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1161,26 +1161,24 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>1.26</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.75</v>
       </c>
       <c r="H20" t="n">
-        <v>1.15</v>
+        <v>1.75</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1188,10 +1186,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1403</v>
+        <v>1350</v>
       </c>
       <c r="D21" t="n">
-        <v>5720</v>
+        <v>5701</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1199,7 +1197,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.65</v>
+        <v>1.68</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1207,7 +1205,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1.45</v>
+        <v>1.15</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1218,7 +1216,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1226,10 +1224,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1366</v>
+        <v>1403</v>
       </c>
       <c r="D22" t="n">
-        <v>5724</v>
+        <v>5720</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1237,24 +1235,26 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="G22" t="n">
-        <v>1.72</v>
+        <v>1.65</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H22" t="n">
-        <v>2.3</v>
+        <v>1.45</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1262,10 +1262,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1304</v>
+        <v>1366</v>
       </c>
       <c r="D23" t="n">
-        <v>5786</v>
+        <v>5724</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1273,13 +1273,13 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.19</v>
+        <v>2.76</v>
       </c>
       <c r="G23" t="n">
-        <v>1.32</v>
+        <v>1.72</v>
       </c>
       <c r="H23" t="n">
-        <v>1.95</v>
+        <v>2.3</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1298,37 +1298,35 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1425</v>
+        <v>1304</v>
       </c>
       <c r="D24" t="n">
-        <v>5809</v>
+        <v>5786</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.19</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1.32</v>
       </c>
       <c r="H24" t="n">
-        <v>0.8</v>
+        <v>1.95</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1336,10 +1334,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1387</v>
+        <v>1425</v>
       </c>
       <c r="D25" t="n">
-        <v>5857</v>
+        <v>5809</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1347,7 +1345,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1.11</v>
+        <v>1.22</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1355,18 +1353,18 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>1.05</v>
+        <v>0.8</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1374,10 +1372,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1365</v>
+        <v>1387</v>
       </c>
       <c r="D26" t="n">
-        <v>5745</v>
+        <v>5857</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1385,24 +1383,26 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="G26" t="n">
-        <v>2.75</v>
+        <v>1.11</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H26" t="n">
-        <v>2.05</v>
+        <v>1.05</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1410,37 +1410,35 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1447</v>
+        <v>1365</v>
       </c>
       <c r="D27" t="n">
-        <v>5623</v>
+        <v>5745</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>4.12</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.75</v>
       </c>
       <c r="H27" t="n">
-        <v>0.5</v>
+        <v>2.05</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1448,18 +1446,18 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1406</v>
+        <v>1447</v>
       </c>
       <c r="D28" t="n">
-        <v>5658</v>
+        <v>5623</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1.35</v>
+        <v>1.51</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1467,7 +1465,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1478,7 +1476,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1486,18 +1484,18 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1350</v>
+        <v>1406</v>
       </c>
       <c r="D29" t="n">
-        <v>5571</v>
+        <v>5658</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1.43</v>
+        <v>1.35</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1505,7 +1503,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.15</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1516,7 +1514,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1524,18 +1522,18 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1390</v>
+        <v>1350</v>
       </c>
       <c r="D30" t="n">
-        <v>5496</v>
+        <v>5571</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1.67</v>
+        <v>1.43</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1543,18 +1541,18 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.06</v>
+        <v>1.15</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1562,10 +1560,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1448</v>
+        <v>1390</v>
       </c>
       <c r="D31" t="n">
-        <v>5583</v>
+        <v>5496</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1573,7 +1571,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1.22</v>
+        <v>1.67</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1581,18 +1579,18 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.04</v>
+        <v>1.06</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1600,35 +1598,37 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1403</v>
+        <v>1448</v>
       </c>
       <c r="D32" t="n">
-        <v>5535</v>
+        <v>5583</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0.93</v>
+        <v>1.22</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H32" t="n">
-        <v>1.74</v>
+        <v>1.04</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1636,26 +1636,24 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1401</v>
+        <v>1403</v>
       </c>
       <c r="D33" t="n">
-        <v>5557</v>
+        <v>5535</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.93</v>
       </c>
       <c r="H33" t="n">
-        <v>1.22</v>
+        <v>1.74</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1666,7 +1664,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1674,18 +1672,18 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1389</v>
+        <v>1401</v>
       </c>
       <c r="D34" t="n">
-        <v>5537</v>
+        <v>5557</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2.03</v>
+        <v>1.08</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1693,7 +1691,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0.75</v>
+        <v>1.22</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1704,7 +1702,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1712,24 +1710,26 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1376</v>
+        <v>1389</v>
       </c>
       <c r="D35" t="n">
-        <v>5577</v>
+        <v>5537</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.93</v>
-      </c>
-      <c r="G35" t="n">
-        <v>1</v>
+        <v>2.03</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H35" t="n">
-        <v>2.2</v>
+        <v>0.75</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1748,10 +1748,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1367</v>
+        <v>1376</v>
       </c>
       <c r="D36" t="n">
-        <v>5516</v>
+        <v>5577</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1759,13 +1759,13 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.07</v>
+        <v>2.93</v>
       </c>
       <c r="G36" t="n">
-        <v>1.94</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1776,7 +1776,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1784,35 +1784,35 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1361</v>
+        <v>1367</v>
       </c>
       <c r="D37" t="n">
-        <v>5532</v>
+        <v>5516</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2.83</v>
+        <v>3.07</v>
       </c>
       <c r="G37" t="n">
-        <v>1.62</v>
+        <v>1.94</v>
       </c>
       <c r="H37" t="n">
-        <v>2.99</v>
+        <v>2.3</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1820,24 +1820,24 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1367</v>
+        <v>1361</v>
       </c>
       <c r="D38" t="n">
-        <v>5581</v>
+        <v>5532</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2.89</v>
+        <v>2.83</v>
       </c>
       <c r="G38" t="n">
-        <v>1.2</v>
+        <v>1.62</v>
       </c>
       <c r="H38" t="n">
-        <v>2.2</v>
+        <v>2.99</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1856,24 +1856,24 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1344</v>
+        <v>1367</v>
       </c>
       <c r="D39" t="n">
-        <v>5530</v>
+        <v>5581</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2.67</v>
+        <v>2.89</v>
       </c>
       <c r="G39" t="n">
-        <v>1.74</v>
+        <v>1.2</v>
       </c>
       <c r="H39" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1892,10 +1892,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1351</v>
+        <v>1344</v>
       </c>
       <c r="D40" t="n">
-        <v>5587</v>
+        <v>5530</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1903,13 +1903,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1.72</v>
+        <v>2.67</v>
       </c>
       <c r="G40" t="n">
-        <v>0.82</v>
+        <v>1.74</v>
       </c>
       <c r="H40" t="n">
-        <v>1.88</v>
+        <v>2.5</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1928,24 +1928,24 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1362</v>
+        <v>1351</v>
       </c>
       <c r="D41" t="n">
-        <v>5606</v>
+        <v>5587</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2.42</v>
+        <v>1.72</v>
       </c>
       <c r="G41" t="n">
-        <v>1.33</v>
+        <v>0.82</v>
       </c>
       <c r="H41" t="n">
-        <v>1.98</v>
+        <v>1.88</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1964,35 +1964,35 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1368</v>
+        <v>1362</v>
       </c>
       <c r="D42" t="n">
-        <v>5688</v>
+        <v>5606</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.57</v>
+        <v>2.42</v>
       </c>
       <c r="G42" t="n">
-        <v>2.25</v>
+        <v>1.33</v>
       </c>
       <c r="H42" t="n">
-        <v>2.85</v>
+        <v>1.98</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2000,35 +2000,35 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="D43" t="n">
-        <v>5610</v>
+        <v>5688</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>4.61</v>
+        <v>3.57</v>
       </c>
       <c r="G43" t="n">
-        <v>4.29</v>
+        <v>2.25</v>
       </c>
       <c r="H43" t="n">
-        <v>3.1</v>
+        <v>2.85</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2036,35 +2036,35 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1335</v>
+        <v>1366</v>
       </c>
       <c r="D44" t="n">
-        <v>5624</v>
+        <v>5610</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>6.65</v>
+        <v>4.61</v>
       </c>
       <c r="G44" t="n">
-        <v>5.3</v>
+        <v>4.29</v>
       </c>
       <c r="H44" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2072,35 +2072,35 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1347</v>
+        <v>1335</v>
       </c>
       <c r="D45" t="n">
-        <v>5609</v>
+        <v>5624</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>4.39</v>
+        <v>6.65</v>
       </c>
       <c r="G45" t="n">
-        <v>3.25</v>
+        <v>5.3</v>
       </c>
       <c r="H45" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2108,35 +2108,35 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1317</v>
+        <v>1347</v>
       </c>
       <c r="D46" t="n">
-        <v>5612</v>
+        <v>5609</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.81</v>
+        <v>4.39</v>
       </c>
       <c r="G46" t="n">
-        <v>2.38</v>
+        <v>3.25</v>
       </c>
       <c r="H46" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2144,37 +2144,35 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1352</v>
+        <v>1317</v>
       </c>
       <c r="D47" t="n">
-        <v>5580</v>
+        <v>5612</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>4.81</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2.38</v>
       </c>
       <c r="H47" t="n">
-        <v>1.05</v>
+        <v>2.5</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2182,35 +2180,37 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1340</v>
+        <v>1352</v>
       </c>
       <c r="D48" t="n">
-        <v>5576</v>
+        <v>5580</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="G48" t="n">
-        <v>1.81</v>
+        <v>1.35</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H48" t="n">
-        <v>2.3</v>
+        <v>1.05</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2218,26 +2218,24 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1323</v>
+        <v>1340</v>
       </c>
       <c r="D49" t="n">
-        <v>5519</v>
+        <v>5576</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.39</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.81</v>
       </c>
       <c r="H49" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.3</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2248,7 +2246,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2256,18 +2254,18 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1316</v>
+        <v>1323</v>
       </c>
       <c r="D50" t="n">
-        <v>5555</v>
+        <v>5519</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1.01</v>
+        <v>1.53</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2275,18 +2273,18 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>0.83</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -2294,35 +2292,37 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1285</v>
+        <v>1316</v>
       </c>
       <c r="D51" t="n">
-        <v>5601</v>
+        <v>5555</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="G51" t="n">
-        <v>0.58</v>
+        <v>1.01</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H51" t="n">
-        <v>1.6</v>
+        <v>0.83</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2330,10 +2330,10 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1281</v>
+        <v>1285</v>
       </c>
       <c r="D52" t="n">
-        <v>5637</v>
+        <v>5601</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2341,13 +2341,13 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1.59</v>
+        <v>1.63</v>
       </c>
       <c r="G52" t="n">
-        <v>0.59</v>
+        <v>0.58</v>
       </c>
       <c r="H52" t="n">
-        <v>1.55</v>
+        <v>1.6</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2366,24 +2366,24 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1260</v>
+        <v>1281</v>
       </c>
       <c r="D53" t="n">
-        <v>5760</v>
+        <v>5637</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>3.14</v>
+        <v>1.59</v>
       </c>
       <c r="G53" t="n">
-        <v>1.95</v>
+        <v>0.59</v>
       </c>
       <c r="H53" t="n">
-        <v>3.05</v>
+        <v>1.55</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -2394,7 +2394,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2402,39 +2402,35 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1352</v>
+        <v>1260</v>
       </c>
       <c r="D54" t="n">
-        <v>5620</v>
+        <v>5760</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>3.44</v>
+        <v>3.14</v>
       </c>
       <c r="G54" t="n">
-        <v>1.76</v>
+        <v>1.95</v>
       </c>
       <c r="H54" t="n">
-        <v>3.1</v>
+        <v>3.05</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>growing off 6cm base</t>
-        </is>
-      </c>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -2442,37 +2438,39 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1405</v>
+        <v>1352</v>
       </c>
       <c r="D55" t="n">
-        <v>5632</v>
+        <v>5620</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>3.44</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1.76</v>
       </c>
       <c r="H55" t="n">
-        <v>0.5</v>
+        <v>3.1</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>growing off 6cm base</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -2480,35 +2478,37 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1288</v>
+        <v>1405</v>
       </c>
       <c r="D56" t="n">
-        <v>5536</v>
+        <v>5632</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="G56" t="n">
-        <v>0.54</v>
+        <v>1.03</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H56" t="n">
-        <v>1.45</v>
+        <v>0.5</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -2516,71 +2516,71 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1251</v>
+        <v>1288</v>
       </c>
       <c r="D57" t="n">
-        <v>5601</v>
+        <v>5536</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>8.300000000000001</v>
+        <v>1.78</v>
       </c>
       <c r="G57" t="n">
-        <v>6.34</v>
+        <v>0.54</v>
       </c>
       <c r="H57" t="n">
-        <v>4.6</v>
+        <v>1.45</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="C58" t="n">
         <v>1251</v>
       </c>
       <c r="D58" t="n">
-        <v>5625</v>
+        <v>5601</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>2.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G58" t="n">
-        <v>1.82</v>
+        <v>6.34</v>
       </c>
       <c r="H58" t="n">
-        <v>1.5</v>
+        <v>4.6</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -2588,26 +2588,24 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1256</v>
+        <v>1251</v>
       </c>
       <c r="D59" t="n">
-        <v>5682</v>
+        <v>5625</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.2</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1.82</v>
       </c>
       <c r="H59" t="n">
-        <v>1.35</v>
+        <v>1.5</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -2618,7 +2616,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -2626,18 +2624,18 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1250</v>
+        <v>1256</v>
       </c>
       <c r="D60" t="n">
-        <v>5720</v>
+        <v>5682</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>1.07</v>
+        <v>1.4</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2645,7 +2643,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1.2</v>
+        <v>1.35</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -2656,7 +2654,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2664,18 +2662,18 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1220</v>
+        <v>1250</v>
       </c>
       <c r="D61" t="n">
-        <v>5642</v>
+        <v>5720</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>1.62</v>
+        <v>1.07</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2683,22 +2681,18 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>0.86</v>
+        <v>1.2</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>3 dead stems</t>
-        </is>
-      </c>
+      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -2706,18 +2700,18 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1272</v>
+        <v>1220</v>
       </c>
       <c r="D62" t="n">
-        <v>5738</v>
+        <v>5642</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>1.34</v>
+        <v>1.62</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2725,18 +2719,22 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>3 dead stems</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -2744,18 +2742,18 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1051</v>
+        <v>1272</v>
       </c>
       <c r="D63" t="n">
-        <v>5842</v>
+        <v>5738</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.47</v>
+        <v>1.34</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2763,7 +2761,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>1.06</v>
+        <v>0.9</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -2774,7 +2772,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -2782,14 +2780,14 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1076</v>
+        <v>1051</v>
       </c>
       <c r="D64" t="n">
-        <v>5838</v>
+        <v>5842</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -2801,7 +2799,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>0.61</v>
+        <v>1.06</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -2812,7 +2810,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -2820,18 +2818,18 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1099</v>
+        <v>1076</v>
       </c>
       <c r="D65" t="n">
-        <v>5794</v>
+        <v>5838</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1.25</v>
+        <v>1.47</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2839,7 +2837,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0.72</v>
+        <v>0.61</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -2850,7 +2848,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -2858,26 +2856,26 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1086</v>
+        <v>1099</v>
       </c>
       <c r="D66" t="n">
-        <v>5771</v>
+        <v>5794</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F66" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
         <v>0.72</v>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H66" t="n">
-        <v>0.54</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
@@ -2888,7 +2886,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2896,10 +2894,10 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1185</v>
+        <v>1086</v>
       </c>
       <c r="D67" t="n">
-        <v>5656</v>
+        <v>5771</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2907,7 +2905,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0.85</v>
+        <v>0.72</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2915,22 +2913,18 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>0.62</v>
+        <v>0.54</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>2 dead stems</t>
-        </is>
-      </c>
+      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -2938,35 +2932,41 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1162</v>
+        <v>1185</v>
       </c>
       <c r="D68" t="n">
-        <v>5626</v>
+        <v>5656</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>4.86</v>
-      </c>
-      <c r="G68" t="n">
-        <v>1.84</v>
+        <v>0.85</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H68" t="n">
-        <v>2.7</v>
+        <v>0.62</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2 dead stems</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -2974,24 +2974,24 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1154</v>
+        <v>1162</v>
       </c>
       <c r="D69" t="n">
-        <v>5564</v>
+        <v>5626</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>5.56</v>
+        <v>4.86</v>
       </c>
       <c r="G69" t="n">
-        <v>3.4</v>
+        <v>1.84</v>
       </c>
       <c r="H69" t="n">
-        <v>4.27</v>
+        <v>2.7</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -3010,24 +3010,24 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1142</v>
+        <v>1154</v>
       </c>
       <c r="D70" t="n">
-        <v>5574</v>
+        <v>5564</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>5.63</v>
+        <v>5.56</v>
       </c>
       <c r="G70" t="n">
-        <v>2.46</v>
+        <v>3.4</v>
       </c>
       <c r="H70" t="n">
-        <v>4.16</v>
+        <v>4.27</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -3038,7 +3038,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -3046,24 +3046,24 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="D71" t="n">
-        <v>5588</v>
+        <v>5574</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>10.6</v>
+        <v>5.63</v>
       </c>
       <c r="G71" t="n">
-        <v>9.199999999999999</v>
+        <v>2.46</v>
       </c>
       <c r="H71" t="n">
-        <v>4.6</v>
+        <v>4.16</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
@@ -3074,7 +3074,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -3082,10 +3082,10 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1142</v>
+        <v>1144</v>
       </c>
       <c r="D72" t="n">
-        <v>5563</v>
+        <v>5588</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3093,28 +3093,24 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>6.76</v>
+        <v>10.6</v>
       </c>
       <c r="G72" t="n">
-        <v>5.28</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H72" t="n">
-        <v>4.68</v>
+        <v>4.6</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>1 dead stem</t>
-        </is>
-      </c>
+      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -3122,35 +3118,39 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1132</v>
+        <v>1142</v>
       </c>
       <c r="D73" t="n">
-        <v>5582</v>
+        <v>5563</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>4.47</v>
+        <v>6.76</v>
       </c>
       <c r="G73" t="n">
-        <v>4.09</v>
+        <v>5.28</v>
       </c>
       <c r="H73" t="n">
-        <v>4.33</v>
+        <v>4.68</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>1 dead stem</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -3158,71 +3158,107 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1116</v>
+        <v>1132</v>
       </c>
       <c r="D74" t="n">
-        <v>5641</v>
+        <v>5582</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>8.91</v>
+        <v>4.47</v>
       </c>
       <c r="G74" t="n">
-        <v>6.01</v>
+        <v>4.09</v>
       </c>
       <c r="H74" t="n">
-        <v>4.79</v>
+        <v>4.33</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>6 dead stems</t>
-        </is>
-      </c>
+      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>1116</v>
+      </c>
+      <c r="D75" t="n">
+        <v>5641</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="G75" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="H75" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>6 dead stems</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
         <v>74</v>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>2025-06</t>
         </is>
       </c>
-      <c r="C75" t="n">
+      <c r="C76" t="n">
         <v>1129</v>
       </c>
-      <c r="D75" t="n">
+      <c r="D76" t="n">
         <v>5600</v>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F75" t="n">
+      <c r="F76" t="n">
         <v>4.34</v>
       </c>
-      <c r="G75" t="n">
+      <c r="G76" t="n">
         <v>2.19</v>
       </c>
-      <c r="H75" t="n">
+      <c r="H76" t="n">
         <v>3.21</v>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I76" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Backup before GIS-style visual redesign.
Captures sex-color markers, legend toggle, PCA juvenile key, and related UI polish.
</commit_message>
<xml_diff>
--- a/Spicebush.xlsx
+++ b/Spicebush.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,32 +558,32 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1480</v>
+        <v>1522</v>
       </c>
       <c r="D4" t="n">
-        <v>6012</v>
+        <v>6036</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>2.51</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>2.38</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -594,7 +594,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -602,24 +602,24 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1522</v>
+        <v>1530</v>
       </c>
       <c r="D5" t="n">
-        <v>6036</v>
+        <v>6005</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.51</v>
+        <v>3.18</v>
       </c>
       <c r="G5" t="n">
-        <v>2.38</v>
+        <v>2.11</v>
       </c>
       <c r="H5" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -638,35 +638,39 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1530</v>
+        <v>1482</v>
       </c>
       <c r="D6" t="n">
-        <v>6005</v>
+        <v>5968</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.18</v>
+        <v>6.8</v>
       </c>
       <c r="G6" t="n">
-        <v>2.11</v>
+        <v>3.7</v>
       </c>
       <c r="H6" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>also Female</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -674,10 +678,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1482</v>
+        <v>1337</v>
       </c>
       <c r="D7" t="n">
-        <v>5968</v>
+        <v>5908</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -685,28 +689,24 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6.8</v>
+        <v>3.05</v>
       </c>
       <c r="G7" t="n">
-        <v>3.7</v>
+        <v>1.9</v>
       </c>
       <c r="H7" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>also Female</t>
-        </is>
-      </c>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -714,10 +714,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1337</v>
+        <v>1577</v>
       </c>
       <c r="D8" t="n">
-        <v>5908</v>
+        <v>5881</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -725,24 +725,24 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3.05</v>
+        <v>13.5</v>
       </c>
       <c r="G8" t="n">
-        <v>1.9</v>
+        <v>5.9</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>6.1</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -750,35 +750,35 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1577</v>
+        <v>1600</v>
       </c>
       <c r="D9" t="n">
-        <v>5881</v>
+        <v>5860</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>13.5</v>
+        <v>15</v>
       </c>
       <c r="G9" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H9" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -786,35 +786,35 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1600</v>
+        <v>1598</v>
       </c>
       <c r="D10" t="n">
-        <v>5860</v>
+        <v>5907</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>15</v>
+        <v>7.3</v>
       </c>
       <c r="G10" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
       <c r="H10" t="n">
-        <v>5.8</v>
+        <v>4.7</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -822,35 +822,35 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1598</v>
+        <v>1550</v>
       </c>
       <c r="D11" t="n">
-        <v>5907</v>
+        <v>5876</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>7.3</v>
+        <v>8.1</v>
       </c>
       <c r="G11" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="H11" t="n">
-        <v>4.7</v>
+        <v>1.3</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -858,10 +858,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1550</v>
+        <v>1593</v>
       </c>
       <c r="D12" t="n">
-        <v>5876</v>
+        <v>5890</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -869,24 +869,24 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>8.1</v>
+        <v>1.65</v>
       </c>
       <c r="G12" t="n">
-        <v>3.7</v>
+        <v>1.04</v>
       </c>
       <c r="H12" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>U</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1593</v>
+        <v>1526</v>
       </c>
       <c r="D13" t="n">
-        <v>5890</v>
+        <v>5822</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -905,13 +905,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1.65</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>1.04</v>
+        <v>3.7</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7</v>
+        <v>3.6</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -930,35 +930,37 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1526</v>
+        <v>1550</v>
       </c>
       <c r="D14" t="n">
-        <v>5822</v>
+        <v>5873</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="G14" t="n">
-        <v>3.7</v>
+        <v>1.1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H14" t="n">
-        <v>3.6</v>
+        <v>0.45</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -966,18 +968,18 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1550</v>
+        <v>1554</v>
       </c>
       <c r="D15" t="n">
-        <v>5873</v>
+        <v>5837</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -985,7 +987,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.45</v>
+        <v>0.83</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -996,7 +998,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1004,10 +1006,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1554</v>
+        <v>1523</v>
       </c>
       <c r="D16" t="n">
-        <v>5837</v>
+        <v>5844</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1015,26 +1017,24 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>10.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5.9</v>
       </c>
       <c r="H16" t="n">
-        <v>0.83</v>
+        <v>5.1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1042,10 +1042,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1523</v>
+        <v>1518</v>
       </c>
       <c r="D17" t="n">
-        <v>5844</v>
+        <v>5865</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1053,24 +1053,24 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>10.5</v>
+        <v>7.25</v>
       </c>
       <c r="G17" t="n">
-        <v>5.9</v>
+        <v>5.4</v>
       </c>
       <c r="H17" t="n">
-        <v>5.1</v>
+        <v>5.03</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1078,35 +1078,35 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1518</v>
+        <v>1458</v>
       </c>
       <c r="D18" t="n">
-        <v>5865</v>
+        <v>5809</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>7.25</v>
+        <v>1.61</v>
       </c>
       <c r="G18" t="n">
-        <v>5.4</v>
+        <v>0.4</v>
       </c>
       <c r="H18" t="n">
-        <v>5.03</v>
+        <v>1.25</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1114,24 +1114,24 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1458</v>
+        <v>1398</v>
       </c>
       <c r="D19" t="n">
-        <v>5809</v>
+        <v>5870</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.61</v>
+        <v>1.26</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4</v>
+        <v>0.75</v>
       </c>
       <c r="H19" t="n">
-        <v>1.25</v>
+        <v>1.75</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1142,7 +1142,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1150,10 +1150,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1398</v>
+        <v>1350</v>
       </c>
       <c r="D20" t="n">
-        <v>5870</v>
+        <v>5701</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1161,24 +1161,26 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.75</v>
+        <v>1.68</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H20" t="n">
-        <v>1.75</v>
+        <v>1.15</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1186,10 +1188,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1350</v>
+        <v>1403</v>
       </c>
       <c r="D21" t="n">
-        <v>5701</v>
+        <v>5720</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1197,7 +1199,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.68</v>
+        <v>1.65</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1205,7 +1207,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1.15</v>
+        <v>1.45</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1216,7 +1218,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1224,10 +1226,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1403</v>
+        <v>1366</v>
       </c>
       <c r="D22" t="n">
-        <v>5720</v>
+        <v>5724</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1235,26 +1237,24 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.76</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1.72</v>
       </c>
       <c r="H22" t="n">
-        <v>1.45</v>
+        <v>2.3</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1262,10 +1262,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1366</v>
+        <v>1304</v>
       </c>
       <c r="D23" t="n">
-        <v>5724</v>
+        <v>5786</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1273,13 +1273,13 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.76</v>
+        <v>2.19</v>
       </c>
       <c r="G23" t="n">
-        <v>1.72</v>
+        <v>1.32</v>
       </c>
       <c r="H23" t="n">
-        <v>2.3</v>
+        <v>1.95</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1298,35 +1298,37 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1304</v>
+        <v>1425</v>
       </c>
       <c r="D24" t="n">
-        <v>5786</v>
+        <v>5809</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="G24" t="n">
-        <v>1.32</v>
+        <v>1.22</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H24" t="n">
-        <v>1.95</v>
+        <v>0.8</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1334,10 +1336,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1425</v>
+        <v>1387</v>
       </c>
       <c r="D25" t="n">
-        <v>5809</v>
+        <v>5857</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1345,7 +1347,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1.22</v>
+        <v>1.11</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1353,18 +1355,18 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.8</v>
+        <v>1.05</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1372,10 +1374,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1387</v>
+        <v>1365</v>
       </c>
       <c r="D26" t="n">
-        <v>5857</v>
+        <v>5745</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1383,26 +1385,24 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>4.12</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2.75</v>
       </c>
       <c r="H26" t="n">
-        <v>1.05</v>
+        <v>2.05</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1410,35 +1410,37 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1365</v>
+        <v>1447</v>
       </c>
       <c r="D27" t="n">
-        <v>5745</v>
+        <v>5623</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="G27" t="n">
-        <v>2.75</v>
+        <v>1.51</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H27" t="n">
-        <v>2.05</v>
+        <v>0.5</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1446,18 +1448,18 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1447</v>
+        <v>1406</v>
       </c>
       <c r="D28" t="n">
-        <v>5623</v>
+        <v>5658</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1.51</v>
+        <v>1.35</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1465,7 +1467,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.5</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1476,7 +1478,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1484,18 +1486,18 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1406</v>
+        <v>1350</v>
       </c>
       <c r="D29" t="n">
-        <v>5658</v>
+        <v>5571</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1.35</v>
+        <v>1.43</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1503,7 +1505,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.15</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1514,7 +1516,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1522,18 +1524,18 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1350</v>
+        <v>1390</v>
       </c>
       <c r="D30" t="n">
-        <v>5571</v>
+        <v>5496</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1.43</v>
+        <v>1.67</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1541,18 +1543,18 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.15</v>
+        <v>1.06</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1560,10 +1562,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1390</v>
+        <v>1448</v>
       </c>
       <c r="D31" t="n">
-        <v>5496</v>
+        <v>5583</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1571,7 +1573,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1.67</v>
+        <v>1.22</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1579,18 +1581,18 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.06</v>
+        <v>1.04</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1598,37 +1600,35 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1448</v>
+        <v>1403</v>
       </c>
       <c r="D32" t="n">
-        <v>5583</v>
+        <v>5535</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.93</v>
       </c>
       <c r="H32" t="n">
-        <v>1.04</v>
+        <v>1.74</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1636,24 +1636,26 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1403</v>
+        <v>1401</v>
       </c>
       <c r="D33" t="n">
-        <v>5535</v>
+        <v>5557</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0.93</v>
+        <v>1.08</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H33" t="n">
-        <v>1.74</v>
+        <v>1.22</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1664,7 +1666,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1672,18 +1674,18 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1401</v>
+        <v>1389</v>
       </c>
       <c r="D34" t="n">
-        <v>5557</v>
+        <v>5537</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1.08</v>
+        <v>2.03</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1691,7 +1693,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1.22</v>
+        <v>0.75</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1702,7 +1704,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1710,26 +1712,24 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1389</v>
+        <v>1376</v>
       </c>
       <c r="D35" t="n">
-        <v>5537</v>
+        <v>5577</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.93</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>0.75</v>
+        <v>2.2</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1748,10 +1748,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1376</v>
+        <v>1367</v>
       </c>
       <c r="D36" t="n">
-        <v>5577</v>
+        <v>5516</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1759,13 +1759,13 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.93</v>
+        <v>3.07</v>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>1.94</v>
       </c>
       <c r="H36" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1776,7 +1776,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1784,35 +1784,35 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1367</v>
+        <v>1361</v>
       </c>
       <c r="D37" t="n">
-        <v>5516</v>
+        <v>5532</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.07</v>
+        <v>2.83</v>
       </c>
       <c r="G37" t="n">
-        <v>1.94</v>
+        <v>1.62</v>
       </c>
       <c r="H37" t="n">
-        <v>2.3</v>
+        <v>2.99</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1820,24 +1820,24 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1361</v>
+        <v>1367</v>
       </c>
       <c r="D38" t="n">
-        <v>5532</v>
+        <v>5581</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2.83</v>
+        <v>2.89</v>
       </c>
       <c r="G38" t="n">
-        <v>1.62</v>
+        <v>1.2</v>
       </c>
       <c r="H38" t="n">
-        <v>2.99</v>
+        <v>2.2</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1856,24 +1856,24 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1367</v>
+        <v>1344</v>
       </c>
       <c r="D39" t="n">
-        <v>5581</v>
+        <v>5530</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2.89</v>
+        <v>2.67</v>
       </c>
       <c r="G39" t="n">
-        <v>1.2</v>
+        <v>1.74</v>
       </c>
       <c r="H39" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1892,10 +1892,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1344</v>
+        <v>1351</v>
       </c>
       <c r="D40" t="n">
-        <v>5530</v>
+        <v>5587</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1903,13 +1903,13 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2.67</v>
+        <v>1.72</v>
       </c>
       <c r="G40" t="n">
-        <v>1.74</v>
+        <v>0.82</v>
       </c>
       <c r="H40" t="n">
-        <v>2.5</v>
+        <v>1.88</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1928,24 +1928,24 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1351</v>
+        <v>1362</v>
       </c>
       <c r="D41" t="n">
-        <v>5587</v>
+        <v>5606</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1.72</v>
+        <v>2.42</v>
       </c>
       <c r="G41" t="n">
-        <v>0.82</v>
+        <v>1.33</v>
       </c>
       <c r="H41" t="n">
-        <v>1.88</v>
+        <v>1.98</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1964,35 +1964,35 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1362</v>
+        <v>1368</v>
       </c>
       <c r="D42" t="n">
-        <v>5606</v>
+        <v>5688</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>2.42</v>
+        <v>3.57</v>
       </c>
       <c r="G42" t="n">
-        <v>1.33</v>
+        <v>2.25</v>
       </c>
       <c r="H42" t="n">
-        <v>1.98</v>
+        <v>2.85</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2000,35 +2000,35 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="D43" t="n">
-        <v>5688</v>
+        <v>5610</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.57</v>
+        <v>4.61</v>
       </c>
       <c r="G43" t="n">
-        <v>2.25</v>
+        <v>4.29</v>
       </c>
       <c r="H43" t="n">
-        <v>2.85</v>
+        <v>3.1</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2036,35 +2036,35 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1366</v>
+        <v>1335</v>
       </c>
       <c r="D44" t="n">
-        <v>5610</v>
+        <v>5624</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>4.61</v>
+        <v>6.65</v>
       </c>
       <c r="G44" t="n">
-        <v>4.29</v>
+        <v>5.3</v>
       </c>
       <c r="H44" t="n">
-        <v>3.1</v>
+        <v>2.6</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2072,35 +2072,35 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1335</v>
+        <v>1347</v>
       </c>
       <c r="D45" t="n">
-        <v>5624</v>
+        <v>5609</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>6.65</v>
+        <v>4.39</v>
       </c>
       <c r="G45" t="n">
-        <v>5.3</v>
+        <v>3.25</v>
       </c>
       <c r="H45" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2108,35 +2108,35 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1347</v>
+        <v>1317</v>
       </c>
       <c r="D46" t="n">
-        <v>5609</v>
+        <v>5612</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.39</v>
+        <v>4.81</v>
       </c>
       <c r="G46" t="n">
-        <v>3.25</v>
+        <v>2.38</v>
       </c>
       <c r="H46" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2144,35 +2144,37 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1317</v>
+        <v>1352</v>
       </c>
       <c r="D47" t="n">
-        <v>5612</v>
+        <v>5580</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>4.81</v>
-      </c>
-      <c r="G47" t="n">
-        <v>2.38</v>
+        <v>1.35</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H47" t="n">
-        <v>2.5</v>
+        <v>1.05</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2180,37 +2182,35 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1352</v>
+        <v>1340</v>
       </c>
       <c r="D48" t="n">
-        <v>5580</v>
+        <v>5576</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>2.39</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1.81</v>
       </c>
       <c r="H48" t="n">
-        <v>1.05</v>
+        <v>2.3</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2218,24 +2218,26 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1340</v>
+        <v>1323</v>
       </c>
       <c r="D49" t="n">
-        <v>5576</v>
+        <v>5519</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="G49" t="n">
-        <v>1.81</v>
+        <v>1.53</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H49" t="n">
-        <v>2.3</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2246,7 +2248,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2254,18 +2256,18 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1323</v>
+        <v>1316</v>
       </c>
       <c r="D50" t="n">
-        <v>5519</v>
+        <v>5555</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1.53</v>
+        <v>1.01</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2273,18 +2275,18 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.83</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -2292,37 +2294,35 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1316</v>
+        <v>1285</v>
       </c>
       <c r="D51" t="n">
-        <v>5555</v>
+        <v>5601</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>1.63</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.58</v>
       </c>
       <c r="H51" t="n">
-        <v>0.83</v>
+        <v>1.6</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2330,10 +2330,10 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1285</v>
+        <v>1281</v>
       </c>
       <c r="D52" t="n">
-        <v>5601</v>
+        <v>5637</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2341,13 +2341,13 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1.63</v>
+        <v>1.59</v>
       </c>
       <c r="G52" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="H52" t="n">
-        <v>1.6</v>
+        <v>1.55</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -2358,7 +2358,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2366,24 +2366,24 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1281</v>
+        <v>1260</v>
       </c>
       <c r="D53" t="n">
-        <v>5637</v>
+        <v>5760</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1.59</v>
+        <v>3.14</v>
       </c>
       <c r="G53" t="n">
-        <v>0.59</v>
+        <v>1.95</v>
       </c>
       <c r="H53" t="n">
-        <v>1.55</v>
+        <v>3.05</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -2394,7 +2394,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2402,35 +2402,39 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1260</v>
+        <v>1352</v>
       </c>
       <c r="D54" t="n">
-        <v>5760</v>
+        <v>5620</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>3.14</v>
+        <v>3.44</v>
       </c>
       <c r="G54" t="n">
-        <v>1.95</v>
+        <v>1.76</v>
       </c>
       <c r="H54" t="n">
-        <v>3.05</v>
+        <v>3.1</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>growing off 6cm base</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -2438,39 +2442,37 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1352</v>
+        <v>1405</v>
       </c>
       <c r="D55" t="n">
-        <v>5620</v>
+        <v>5632</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>3.44</v>
-      </c>
-      <c r="G55" t="n">
-        <v>1.76</v>
+        <v>1.03</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H55" t="n">
-        <v>3.1</v>
+        <v>0.5</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>growing off 6cm base</t>
-        </is>
-      </c>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -2478,37 +2480,35 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1405</v>
+        <v>1288</v>
       </c>
       <c r="D56" t="n">
-        <v>5632</v>
+        <v>5536</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>1.78</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.54</v>
       </c>
       <c r="H56" t="n">
-        <v>0.5</v>
+        <v>1.45</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -2516,71 +2516,71 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1288</v>
+        <v>1251</v>
       </c>
       <c r="D57" t="n">
-        <v>5536</v>
+        <v>5601</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>1.78</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G57" t="n">
-        <v>0.54</v>
+        <v>6.34</v>
       </c>
       <c r="H57" t="n">
-        <v>1.45</v>
+        <v>4.6</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="C58" t="n">
         <v>1251</v>
       </c>
       <c r="D58" t="n">
-        <v>5601</v>
+        <v>5625</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>8.300000000000001</v>
+        <v>2.2</v>
       </c>
       <c r="G58" t="n">
-        <v>6.34</v>
+        <v>1.82</v>
       </c>
       <c r="H58" t="n">
-        <v>4.6</v>
+        <v>1.5</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>U</t>
         </is>
       </c>
       <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -2588,24 +2588,26 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1251</v>
+        <v>1256</v>
       </c>
       <c r="D59" t="n">
-        <v>5625</v>
+        <v>5682</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="G59" t="n">
-        <v>1.82</v>
+        <v>1.4</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="H59" t="n">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -2616,7 +2618,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -2624,18 +2626,18 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1256</v>
+        <v>1250</v>
       </c>
       <c r="D60" t="n">
-        <v>5682</v>
+        <v>5720</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>1.4</v>
+        <v>1.07</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2643,7 +2645,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1.35</v>
+        <v>1.2</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -2654,7 +2656,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2662,18 +2664,18 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1250</v>
+        <v>1220</v>
       </c>
       <c r="D61" t="n">
-        <v>5720</v>
+        <v>5642</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>1.07</v>
+        <v>1.62</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2681,18 +2683,22 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.2</v>
+        <v>0.86</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>3 dead stems</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -2700,18 +2706,18 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1220</v>
+        <v>1272</v>
       </c>
       <c r="D62" t="n">
-        <v>5642</v>
+        <v>5738</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>1.62</v>
+        <v>1.34</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2719,22 +2725,18 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>3 dead stems</t>
-        </is>
-      </c>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -2742,18 +2744,18 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1272</v>
+        <v>1051</v>
       </c>
       <c r="D63" t="n">
-        <v>5738</v>
+        <v>5842</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1.34</v>
+        <v>1.47</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2761,7 +2763,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>0.9</v>
+        <v>1.06</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -2772,7 +2774,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -2780,14 +2782,14 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1051</v>
+        <v>1076</v>
       </c>
       <c r="D64" t="n">
-        <v>5842</v>
+        <v>5838</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -2799,7 +2801,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1.06</v>
+        <v>0.61</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -2810,7 +2812,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -2818,18 +2820,18 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1076</v>
+        <v>1099</v>
       </c>
       <c r="D65" t="n">
-        <v>5838</v>
+        <v>5794</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1.47</v>
+        <v>1.25</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2837,7 +2839,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0.61</v>
+        <v>0.72</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -2848,7 +2850,7 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -2856,18 +2858,18 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1099</v>
+        <v>1086</v>
       </c>
       <c r="D66" t="n">
-        <v>5794</v>
+        <v>5771</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>1.25</v>
+        <v>0.72</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2875,7 +2877,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>0.72</v>
+        <v>0.54</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
@@ -2886,7 +2888,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2894,10 +2896,10 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1086</v>
+        <v>1185</v>
       </c>
       <c r="D67" t="n">
-        <v>5771</v>
+        <v>5656</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2905,7 +2907,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0.72</v>
+        <v>0.85</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2913,18 +2915,22 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>0.54</v>
+        <v>0.62</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2 dead stems</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -2932,41 +2938,35 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1185</v>
+        <v>1162</v>
       </c>
       <c r="D68" t="n">
-        <v>5656</v>
+        <v>5626</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>4.86</v>
+      </c>
+      <c r="G68" t="n">
+        <v>1.84</v>
       </c>
       <c r="H68" t="n">
-        <v>0.62</v>
+        <v>2.7</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>2 dead stems</t>
-        </is>
-      </c>
+      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -2974,24 +2974,24 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1162</v>
+        <v>1154</v>
       </c>
       <c r="D69" t="n">
-        <v>5626</v>
+        <v>5564</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>4.86</v>
+        <v>5.56</v>
       </c>
       <c r="G69" t="n">
-        <v>1.84</v>
+        <v>3.4</v>
       </c>
       <c r="H69" t="n">
-        <v>2.7</v>
+        <v>4.27</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -3010,24 +3010,24 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1154</v>
+        <v>1142</v>
       </c>
       <c r="D70" t="n">
-        <v>5564</v>
+        <v>5574</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>5.56</v>
+        <v>5.63</v>
       </c>
       <c r="G70" t="n">
-        <v>3.4</v>
+        <v>2.46</v>
       </c>
       <c r="H70" t="n">
-        <v>4.27</v>
+        <v>4.16</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -3038,7 +3038,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -3046,24 +3046,24 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1142</v>
+        <v>1144</v>
       </c>
       <c r="D71" t="n">
-        <v>5574</v>
+        <v>5588</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>5.63</v>
+        <v>10.6</v>
       </c>
       <c r="G71" t="n">
-        <v>2.46</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H71" t="n">
-        <v>4.16</v>
+        <v>4.6</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
@@ -3074,7 +3074,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -3082,10 +3082,10 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="D72" t="n">
-        <v>5588</v>
+        <v>5563</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3093,24 +3093,28 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>10.6</v>
+        <v>6.76</v>
       </c>
       <c r="G72" t="n">
-        <v>9.199999999999999</v>
+        <v>5.28</v>
       </c>
       <c r="H72" t="n">
-        <v>4.6</v>
+        <v>4.68</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>1 dead stem</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -3118,39 +3122,35 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1142</v>
+        <v>1132</v>
       </c>
       <c r="D73" t="n">
-        <v>5563</v>
+        <v>5582</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>6.76</v>
+        <v>4.47</v>
       </c>
       <c r="G73" t="n">
-        <v>5.28</v>
+        <v>4.09</v>
       </c>
       <c r="H73" t="n">
-        <v>4.68</v>
+        <v>4.33</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>1 dead stem</t>
-        </is>
-      </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -3158,35 +3158,39 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1132</v>
+        <v>1116</v>
       </c>
       <c r="D74" t="n">
-        <v>5582</v>
+        <v>5641</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>4.47</v>
+        <v>8.91</v>
       </c>
       <c r="G74" t="n">
-        <v>4.09</v>
+        <v>6.01</v>
       </c>
       <c r="H74" t="n">
-        <v>4.33</v>
+        <v>4.79</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>6 dead stems</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -3194,71 +3198,31 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1116</v>
+        <v>1129</v>
       </c>
       <c r="D75" t="n">
-        <v>5641</v>
+        <v>5600</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>8.91</v>
+        <v>4.34</v>
       </c>
       <c r="G75" t="n">
-        <v>6.01</v>
+        <v>2.19</v>
       </c>
       <c r="H75" t="n">
-        <v>4.79</v>
+        <v>3.21</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>6 dead stems</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>74</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>1129</v>
-      </c>
-      <c r="D76" t="n">
-        <v>5600</v>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F76" t="n">
-        <v>4.34</v>
-      </c>
-      <c r="G76" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="H76" t="n">
-        <v>3.21</v>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>